<commit_message>
Calculate MAE for contacts/trow
</commit_message>
<xml_diff>
--- a/sessions/contacts/trow/analysis/doppler_vs_positional.xlsx
+++ b/sessions/contacts/trow/analysis/doppler_vs_positional.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25028"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25128"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\mike\projects\docs\gps-guides\sessions\contacts\will\analysis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mwgeo\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDD024ED-BA6B-4A90-AC23-726DD8FD26F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0A1A5A4-1E3D-4935-AC95-B2245AA040D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{1A0D1499-61F0-4420-A350-725B2B0FF3B8}"/>
   </bookViews>
   <sheets>
     <sheet name="vertix-2" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -23,7 +23,9 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
       </xcalcf:calcFeatures>
@@ -33,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
   <si>
     <t>doppler</t>
   </si>
@@ -60,6 +62,9 @@
   </si>
   <si>
     <t>diff</t>
+  </si>
+  <si>
+    <t>abs diff</t>
   </si>
 </sst>
 </file>
@@ -173,7 +178,17 @@
           </a:p>
           <a:p>
             <a:pPr>
-              <a:defRPr/>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
             </a:pPr>
             <a:r>
               <a:rPr lang="en-GB" sz="1200"/>
@@ -1183,13 +1198,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>11</xdr:col>
+      <xdr:col>13</xdr:col>
       <xdr:colOff>19049</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>21</xdr:col>
+      <xdr:col>23</xdr:col>
       <xdr:colOff>352424</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>95250</xdr:rowOff>
@@ -1517,10 +1532,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31D1B82B-501B-496C-BA82-2B77B32B0676}">
-  <dimension ref="A1:J47"/>
+  <dimension ref="A1:K47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>2</v>
       </c>
@@ -1545,8 +1560,11 @@
       <c r="J1" s="3" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K1" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>0.48645833333333338</v>
       </c>
@@ -1573,8 +1591,12 @@
         <f>G2-C2</f>
         <v>-0.13700000000000045</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K2" s="2">
+        <f>ABS(J2)</f>
+        <v>0.13700000000000045</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>0.4878703703703704</v>
       </c>
@@ -1601,8 +1623,12 @@
         <f>G3-C3</f>
         <v>0.13400000000000034</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K3" s="2">
+        <f t="shared" ref="K3:K21" si="1">ABS(J3)</f>
+        <v>0.13400000000000034</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>0.49009259259259258</v>
       </c>
@@ -1629,8 +1655,12 @@
         <f>G4-C4</f>
         <v>0.18900000000000006</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K4" s="2">
+        <f t="shared" si="1"/>
+        <v>0.18900000000000006</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>0.49144675925925929</v>
       </c>
@@ -1653,9 +1683,16 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J5" s="2"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J5" s="2">
+        <f>G5-C5</f>
+        <v>-9.5000000000002416E-2</v>
+      </c>
+      <c r="K5" s="2">
+        <f t="shared" si="1"/>
+        <v>9.5000000000002416E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>0.49373842592592593</v>
       </c>
@@ -1678,9 +1715,16 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J6" s="2"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J6" s="2">
+        <f>G6-C6</f>
+        <v>0.24399999999999977</v>
+      </c>
+      <c r="K6" s="2">
+        <f t="shared" si="1"/>
+        <v>0.24399999999999977</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>0.49849537037037034</v>
       </c>
@@ -1704,11 +1748,15 @@
         <v/>
       </c>
       <c r="J7" s="2">
-        <f t="shared" ref="J7:J21" si="1">G7-C7</f>
+        <f t="shared" ref="J7:J21" si="2">G7-C7</f>
         <v>-5.4999999999999716E-2</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K7" s="2">
+        <f t="shared" si="1"/>
+        <v>5.4999999999999716E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>0.50439814814814821</v>
       </c>
@@ -1732,11 +1780,15 @@
         <v/>
       </c>
       <c r="J8" s="2">
+        <f t="shared" si="2"/>
+        <v>-5.1000000000001933E-2</v>
+      </c>
+      <c r="K8" s="2">
         <f t="shared" si="1"/>
-        <v>-5.1000000000001933E-2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+        <v>5.1000000000001933E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>0.50596064814814812</v>
       </c>
@@ -1760,11 +1812,15 @@
         <v/>
       </c>
       <c r="J9" s="2">
+        <f t="shared" si="2"/>
+        <v>-3.3000000000001251E-2</v>
+      </c>
+      <c r="K9" s="2">
         <f t="shared" si="1"/>
-        <v>-3.3000000000001251E-2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+        <v>3.3000000000001251E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>0.50880787037037034</v>
       </c>
@@ -1788,11 +1844,15 @@
         <v/>
       </c>
       <c r="J10" s="2">
+        <f t="shared" si="2"/>
+        <v>6.4000000000000057E-2</v>
+      </c>
+      <c r="K10" s="2">
         <f t="shared" si="1"/>
         <v>6.4000000000000057E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>0.51107638888888884</v>
       </c>
@@ -1816,11 +1876,15 @@
         <v/>
       </c>
       <c r="J11" s="2">
+        <f t="shared" si="2"/>
+        <v>4.9999999999990052E-3</v>
+      </c>
+      <c r="K11" s="2">
         <f t="shared" si="1"/>
         <v>4.9999999999990052E-3</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>0.52049768518518513</v>
       </c>
@@ -1844,11 +1908,15 @@
         <v/>
       </c>
       <c r="J12" s="2">
+        <f t="shared" si="2"/>
+        <v>6.3000000000002387E-2</v>
+      </c>
+      <c r="K12" s="2">
         <f t="shared" si="1"/>
         <v>6.3000000000002387E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>0.52671296296296299</v>
       </c>
@@ -1872,11 +1940,15 @@
         <v/>
       </c>
       <c r="J13" s="2">
+        <f t="shared" si="2"/>
+        <v>-0.19400000000000261</v>
+      </c>
+      <c r="K13" s="2">
         <f t="shared" si="1"/>
-        <v>-0.19400000000000261</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+        <v>0.19400000000000261</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>0.52900462962962969</v>
       </c>
@@ -1900,11 +1972,15 @@
         <v/>
       </c>
       <c r="J14" s="2">
+        <f t="shared" si="2"/>
+        <v>8.2000000000000739E-2</v>
+      </c>
+      <c r="K14" s="2">
         <f t="shared" si="1"/>
         <v>8.2000000000000739E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>0.56452546296296291</v>
       </c>
@@ -1928,11 +2004,15 @@
         <v/>
       </c>
       <c r="J15" s="2">
+        <f t="shared" si="2"/>
+        <v>3.0999999999998806E-2</v>
+      </c>
+      <c r="K15" s="2">
         <f t="shared" si="1"/>
         <v>3.0999999999998806E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>0.57251157407407405</v>
       </c>
@@ -1956,11 +2036,15 @@
         <v/>
       </c>
       <c r="J16" s="2">
+        <f t="shared" si="2"/>
+        <v>-6.6000000000002501E-2</v>
+      </c>
+      <c r="K16" s="2">
         <f t="shared" si="1"/>
-        <v>-6.6000000000002501E-2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+        <v>6.6000000000002501E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>0.57921296296296299</v>
       </c>
@@ -1984,11 +2068,15 @@
         <v/>
       </c>
       <c r="J17" s="2">
+        <f t="shared" si="2"/>
+        <v>-8.6999999999999744E-2</v>
+      </c>
+      <c r="K17" s="2">
         <f t="shared" si="1"/>
-        <v>-8.6999999999999744E-2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+        <v>8.6999999999999744E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>0.58068287037037036</v>
       </c>
@@ -2012,11 +2100,15 @@
         <v/>
       </c>
       <c r="J18" s="2">
+        <f t="shared" si="2"/>
+        <v>-2.1999999999998465E-2</v>
+      </c>
+      <c r="K18" s="2">
         <f t="shared" si="1"/>
-        <v>-2.1999999999998465E-2</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+        <v>2.1999999999998465E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>0.58280092592592592</v>
       </c>
@@ -2040,11 +2132,15 @@
         <v/>
       </c>
       <c r="J19" s="2">
+        <f t="shared" si="2"/>
+        <v>-6.0999999999999943E-2</v>
+      </c>
+      <c r="K19" s="2">
         <f t="shared" si="1"/>
-        <v>-6.0999999999999943E-2</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+        <v>6.0999999999999943E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>0.58520833333333333</v>
       </c>
@@ -2068,11 +2164,15 @@
         <v/>
       </c>
       <c r="J20" s="2">
+        <f t="shared" si="2"/>
+        <v>0.11599999999999966</v>
+      </c>
+      <c r="K20" s="2">
         <f t="shared" si="1"/>
         <v>0.11599999999999966</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>0.59005787037037039</v>
       </c>
@@ -2096,60 +2196,78 @@
         <v/>
       </c>
       <c r="J21" s="2">
+        <f t="shared" si="2"/>
+        <v>-3.5000000000003695E-2</v>
+      </c>
+      <c r="K21" s="2">
         <f t="shared" si="1"/>
-        <v>-3.5000000000003695E-2</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+        <v>3.5000000000003695E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="J22" s="2"/>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K22" s="2"/>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="H23" t="s">
         <v>4</v>
       </c>
       <c r="J23" s="2">
-        <f>MIN($J$2:$J$21)</f>
+        <f>MIN(J$2:J$21)</f>
         <v>-0.19400000000000261</v>
       </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K23" s="2">
+        <f>MIN(K$2:K$21)</f>
+        <v>4.9999999999990052E-3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="H24" t="s">
         <v>5</v>
       </c>
       <c r="J24" s="2">
-        <f>AVERAGE($J$2:$J$21)</f>
-        <v>-3.1666666666671814E-3</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+        <f>AVERAGE(J$2:J$21)</f>
+        <v>4.5999999999994049E-3</v>
+      </c>
+      <c r="K24" s="2">
+        <f>AVERAGE(K$2:K$21)</f>
+        <v>8.8200000000000681E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="H25" t="s">
         <v>6</v>
       </c>
       <c r="J25" s="2">
-        <f>MAX($J$2:$J$21)</f>
-        <v>0.18900000000000006</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+        <f>MAX(J$2:J$21)</f>
+        <v>0.24399999999999977</v>
+      </c>
+      <c r="K25" s="2">
+        <f>MAX(K$2:K$21)</f>
+        <v>0.24399999999999977</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="J26" s="2"/>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K26" s="2"/>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
       <c r="E28" s="1"/>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="1"/>
       <c r="E29" s="1"/>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="1"/>
       <c r="E30" s="1"/>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="1"/>
       <c r="E31" s="1"/>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="1"/>
       <c r="E32" s="1"/>
     </row>
@@ -2218,6 +2336,16 @@
     <sortCondition ref="A28:A47"/>
   </sortState>
   <conditionalFormatting sqref="J2:J21">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color theme="7" tint="0.79998168889431442"/>
+        <color rgb="FFFF0000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K2:K21">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>